<commit_message>
Fix web-apps load-order race (80 AMD modules extend BaseView/Window with define([])) at build time; phone Slides open with the slide strip collapsed (UI toggle + relayout); sales sample: growth formulas instead of an uncached chart; iPad store shots in portrait
Reproduced the race in Chrome (Slides never starts: Common.UI.BaseView undefined in ColorPaletteExt.js);
after declaring the dependencies: 3/3 clean loads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/store/samples/sales_ar.xlsx
+++ b/store/samples/sales_ar.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="6">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,17 @@
       <name val="Cairo"/>
       <b val="1"/>
       <color rgb="00154F5E"/>
+    </font>
+    <font>
+      <name val="Cairo"/>
+      <b val="1"/>
+      <color rgb="001B8A4B"/>
+    </font>
+    <font>
+      <name val="Cairo"/>
+      <b val="1"/>
+      <color rgb="00C88A12"/>
+      <sz val="12"/>
     </font>
   </fonts>
   <fills count="4">
@@ -89,12 +100,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -102,6 +116,9 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -109,9 +126,13 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="9" fontId="6" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -186,163 +207,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <chart>
-    <title>
-      <tx>
-        <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-            <a:pPr>
-              <a:defRPr/>
-            </a:pPr>
-            <a:r>
-              <a:t>المبيعات الشهرية</a:t>
-            </a:r>
-          </a:p>
-        </rich>
-      </tx>
-    </title>
-    <plotArea>
-      <barChart>
-        <barDir val="col"/>
-        <grouping val="clustered"/>
-        <ser>
-          <idx val="0"/>
-          <order val="0"/>
-          <tx>
-            <strRef>
-              <f>'المبيعات'!A4</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'المبيعات'!$B$3:$G$3</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'المبيعات'!$B$4:$G$4</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="1"/>
-          <order val="1"/>
-          <tx>
-            <strRef>
-              <f>'المبيعات'!A5</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'المبيعات'!$B$3:$G$3</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'المبيعات'!$B$5:$G$5</f>
-            </numRef>
-          </val>
-        </ser>
-        <ser>
-          <idx val="2"/>
-          <order val="2"/>
-          <tx>
-            <strRef>
-              <f>'المبيعات'!A6</f>
-            </strRef>
-          </tx>
-          <spPr>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-              <a:prstDash val="solid"/>
-            </a:ln>
-          </spPr>
-          <cat>
-            <numRef>
-              <f>'المبيعات'!$B$3:$G$3</f>
-            </numRef>
-          </cat>
-          <val>
-            <numRef>
-              <f>'المبيعات'!$B$6:$G$6</f>
-            </numRef>
-          </val>
-        </ser>
-        <gapWidth val="150"/>
-        <axId val="10"/>
-        <axId val="100"/>
-      </barChart>
-      <catAx>
-        <axId val="10"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="100"/>
-        <lblOffset val="100"/>
-      </catAx>
-      <valAx>
-        <axId val="100"/>
-        <scaling>
-          <orientation val="minMax"/>
-        </scaling>
-        <axPos val="l"/>
-        <majorGridlines/>
-        <majorTickMark val="none"/>
-        <minorTickMark val="none"/>
-        <crossAx val="10"/>
-      </valAx>
-    </plotArea>
-    <legend>
-      <legendPos val="r"/>
-    </legend>
-    <plotVisOnly val="1"/>
-    <dispBlanksAs val="gap"/>
-  </chart>
-</chartSpace>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>0</col>
-      <colOff>0</colOff>
-      <row>8</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="5400000" cy="2700000"/>
-    <graphicFrame>
-      <nvGraphicFramePr>
-        <cNvPr id="1" name="Chart 1"/>
-        <cNvGraphicFramePr/>
-      </nvGraphicFramePr>
-      <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
-        </a:graphicData>
-      </a:graphic>
-    </graphicFrame>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -634,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H7"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -645,6 +509,7 @@
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="10" customWidth="1" min="7" max="7"/>
     <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -695,131 +560,158 @@
           <t>الإجمالي</t>
         </is>
       </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>النمو</t>
+        </is>
+      </c>
     </row>
     <row r="4">
-      <c r="A4" s="3" t="inlineStr">
+      <c r="A4" s="4" t="inlineStr">
         <is>
           <t>دبي</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
+      <c r="B4" s="5" t="n">
         <v>312</v>
       </c>
-      <c r="C4" s="4" t="n">
+      <c r="C4" s="5" t="n">
         <v>298</v>
       </c>
-      <c r="D4" s="4" t="n">
+      <c r="D4" s="5" t="n">
         <v>341</v>
       </c>
-      <c r="E4" s="4" t="n">
+      <c r="E4" s="5" t="n">
         <v>365</v>
       </c>
-      <c r="F4" s="4" t="n">
+      <c r="F4" s="5" t="n">
         <v>388</v>
       </c>
-      <c r="G4" s="4" t="n">
+      <c r="G4" s="5" t="n">
         <v>402</v>
       </c>
-      <c r="H4" s="5">
+      <c r="H4" s="6">
         <f>SUM(B4:G4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="7">
+        <f>(G4-B4)/B4</f>
         <v/>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>أبوظبي</t>
         </is>
       </c>
-      <c r="B5" s="7" t="n">
+      <c r="B5" s="9" t="n">
         <v>254</v>
       </c>
-      <c r="C5" s="7" t="n">
+      <c r="C5" s="9" t="n">
         <v>262</v>
       </c>
-      <c r="D5" s="7" t="n">
+      <c r="D5" s="9" t="n">
         <v>271</v>
       </c>
-      <c r="E5" s="7" t="n">
+      <c r="E5" s="9" t="n">
         <v>290</v>
       </c>
-      <c r="F5" s="7" t="n">
+      <c r="F5" s="9" t="n">
         <v>301</v>
       </c>
-      <c r="G5" s="7" t="n">
+      <c r="G5" s="9" t="n">
         <v>318</v>
       </c>
-      <c r="H5" s="8">
+      <c r="H5" s="10">
         <f>SUM(B5:G5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="11">
+        <f>(G5-B5)/B5</f>
         <v/>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="4" t="inlineStr">
         <is>
           <t>الشارقة</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
+      <c r="B6" s="5" t="n">
         <v>98</v>
       </c>
-      <c r="C6" s="4" t="n">
+      <c r="C6" s="5" t="n">
         <v>104</v>
       </c>
-      <c r="D6" s="4" t="n">
+      <c r="D6" s="5" t="n">
         <v>112</v>
       </c>
-      <c r="E6" s="4" t="n">
+      <c r="E6" s="5" t="n">
         <v>121</v>
       </c>
-      <c r="F6" s="4" t="n">
+      <c r="F6" s="5" t="n">
         <v>133</v>
       </c>
-      <c r="G6" s="4" t="n">
+      <c r="G6" s="5" t="n">
         <v>140</v>
       </c>
-      <c r="H6" s="5">
+      <c r="H6" s="6">
         <f>SUM(B6:G6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="7">
+        <f>(G6-B6)/B6</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="4" t="inlineStr">
         <is>
           <t>المجموع</t>
         </is>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="12">
         <f>SUM(B4:B6)</f>
         <v/>
       </c>
-      <c r="C7" s="9">
+      <c r="C7" s="12">
         <f>SUM(C4:C6)</f>
         <v/>
       </c>
-      <c r="D7" s="9">
+      <c r="D7" s="12">
         <f>SUM(D4:D6)</f>
         <v/>
       </c>
-      <c r="E7" s="9">
+      <c r="E7" s="12">
         <f>SUM(E4:E6)</f>
         <v/>
       </c>
-      <c r="F7" s="9">
+      <c r="F7" s="12">
         <f>SUM(F4:F6)</f>
         <v/>
       </c>
-      <c r="G7" s="9">
+      <c r="G7" s="12">
         <f>SUM(G4:G6)</f>
         <v/>
       </c>
-      <c r="H7" s="9">
+      <c r="H7" s="12">
         <f>SUM(H4:H6)</f>
         <v/>
+      </c>
+      <c r="I7" s="7">
+        <f>(G7-B7)/B7</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="13" t="inlineStr">
+        <is>
+          <t>أعلى نمو: الشارقة</t>
+        </is>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>